<commit_message>
additional logic to document changes
</commit_message>
<xml_diff>
--- a/mockData.xlsx
+++ b/mockData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://endava-my.sharepoint.com/personal/dumitru_plamadeala_endava_com/Documents/Desktop/NSG-MRE-SCRIPT/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://endava-my.sharepoint.com/personal/dumitru_plamadeala_endava_com/Documents/Desktop/NSG-MRE-SCRIPT/output/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="243" documentId="13_ncr:1_{7A7F1FDD-8B04-4441-BDD8-5B14B5359350}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{89A4F90A-8126-4736-91A8-517E3E4E0582}"/>
+  <xr:revisionPtr revIDLastSave="298" documentId="13_ncr:1_{7A7F1FDD-8B04-4441-BDD8-5B14B5359350}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EB2078F8-C425-480A-B6E1-03AA51170F21}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{66E66D74-05FB-4940-AC6B-6DDB17CE64BE}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{66E66D74-05FB-4940-AC6B-6DDB17CE64BE}"/>
   </bookViews>
   <sheets>
     <sheet name="CoreRules" sheetId="1" r:id="rId1"/>
@@ -37,15 +37,21 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="73">
   <si>
     <t>Action</t>
   </si>
   <si>
+    <t>Source Host Name (DNS) FQDN</t>
+  </si>
+  <si>
+    <t>Source IP address / Subnet / Range IP</t>
+  </si>
+  <si>
     <t>Destination Host Name (DNS) FQDN</t>
   </si>
   <si>
-    <t>Source Host Name (DNS) FQDN</t>
+    <t>Destination IP address / Subnet / Range IP</t>
   </si>
   <si>
     <t>Destination Protocol</t>
@@ -66,188 +72,296 @@
     <t>Rule Type</t>
   </si>
   <si>
+    <t>Temporary Rule Duration (in Days)</t>
+  </si>
+  <si>
+    <t>BussinesJustification</t>
+  </si>
+  <si>
+    <t>Additional Comments</t>
+  </si>
+  <si>
+    <t>Diff</t>
+  </si>
+  <si>
+    <t>Create</t>
+  </si>
+  <si>
+    <t>CI20</t>
+  </si>
+  <si>
+    <t>200.28.32.12,200.16.20.30,200.16.20.31, 200.16.20.32, 200.16.20.33, 200.16.20.34</t>
+  </si>
+  <si>
+    <t>10.200.0.0/16</t>
+  </si>
+  <si>
+    <t>UDP</t>
+  </si>
+  <si>
+    <t>32914;5872;44109;1023;65500;21345;38901;770-900;49152;12008</t>
+  </si>
+  <si>
+    <t>CORE_Trunk_UDP</t>
+  </si>
+  <si>
+    <t>Permanent</t>
+  </si>
+  <si>
+    <t>CORE parts</t>
+  </si>
+  <si>
+    <t>Update</t>
+  </si>
+  <si>
+    <t>CI40</t>
+  </si>
+  <si>
+    <t>200.28.32.14,200.28.32.15</t>
+  </si>
+  <si>
+    <t>CORE_Fuel_UDP</t>
+  </si>
+  <si>
+    <t>removed: 8000</t>
+  </si>
+  <si>
+    <t>Action: Update
+Changes:
+  DestinationPortRanges:
+    Removed:
+      - '8000'</t>
+  </si>
+  <si>
+    <t>CI50</t>
+  </si>
+  <si>
+    <t>10.101.0.0/17</t>
+  </si>
+  <si>
+    <t>TCP</t>
+  </si>
+  <si>
+    <t>CORE_Speed_TCPPPPP</t>
+  </si>
+  <si>
+    <t>Action: Update
+Changes:
+  SourceAddressPrefixes:
+    Added:
+      - '28.32.15'
+  DestinationAddressPrefixes:
+    Removed:
+      - '10.200.0.0/17'
+    Added:
+      - '10.101.0.0/17'</t>
+  </si>
+  <si>
+    <t>CI1</t>
+  </si>
+  <si>
+    <t>10.28.32.11</t>
+  </si>
+  <si>
+    <t>hostname1.porche.com</t>
+  </si>
+  <si>
+    <t>10.10.10.10, 10.10.10.11, 10.10.10.12</t>
+  </si>
+  <si>
+    <t>443,25;100;101</t>
+  </si>
+  <si>
+    <t>Wheels_P</t>
+  </si>
+  <si>
+    <t>CI1 - Wheel_P</t>
+  </si>
+  <si>
+    <t>CI2</t>
+  </si>
+  <si>
+    <t>10.28.32.12,10.16.20.30,10.16.20.31, 10.16.20.32, 10.16.20.33,10.28.32.12, 10.16.20.34</t>
+  </si>
+  <si>
+    <t>hostname2.porche.com</t>
+  </si>
+  <si>
+    <t>10.10.10.11</t>
+  </si>
+  <si>
+    <t>60421; 1723; 33891; 25000; 49160; 8081; 12345; 53210; 4096; 650</t>
+  </si>
+  <si>
+    <t>Hood_P_I_D</t>
+  </si>
+  <si>
+    <t>CI2 - Hood_P_I_D</t>
+  </si>
+  <si>
+    <t>CI7</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">10.28.32.101; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>10.16.20.34</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">hostname1.porche.com, </t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">10.10.10.14; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>99.99.99</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>433;</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>9999</t>
+    </r>
+  </si>
+  <si>
+    <t>ANOTHER_NAME</t>
+  </si>
+  <si>
+    <t>CI4 - Wheel-New_1</t>
+  </si>
+  <si>
+    <t>Action: Update
+Changes:
+  SourceAddressPrefixes:
+    Added:
+      - '10.16.20.34'
+  DestinationAddressPrefixes:
+    Added:
+      - '99.99.99'
+  DestinationPortRanges:
+    Added:
+      - '9999'</t>
+  </si>
+  <si>
+    <t>CI8</t>
+  </si>
+  <si>
+    <t>100.100.0.10</t>
+  </si>
+  <si>
+    <t>10.10.10.14</t>
+  </si>
+  <si>
+    <t>odie_1508</t>
+  </si>
+  <si>
+    <t>CI5</t>
+  </si>
+  <si>
+    <t>*</t>
+  </si>
+  <si>
+    <t>hostname1.porche.com, hostname2.porche.com, hostname3.porche.com, hostname4.porche.com</t>
+  </si>
+  <si>
+    <t>10.10.10.10, 10.10.10.11, 10.10.10.12, 10.10.10.13, 10.10.10.14, 10.10.10.15</t>
+  </si>
+  <si>
+    <t>CATCH_MISSED_TRAFFIC_TCP</t>
+  </si>
+  <si>
     <t>Temporary</t>
   </si>
   <si>
-    <t>BussinesJustification</t>
-  </si>
-  <si>
-    <t>Additional Comments</t>
-  </si>
-  <si>
-    <t>Create</t>
-  </si>
-  <si>
-    <t>CI1</t>
-  </si>
-  <si>
-    <t>CI2</t>
-  </si>
-  <si>
-    <t>CI5</t>
+    <t>Default Rule to catch Missed Traffic TCP</t>
+  </si>
+  <si>
+    <t>Protection Rule</t>
   </si>
   <si>
     <t>CI6</t>
   </si>
   <si>
-    <t>10.28.32.11</t>
-  </si>
-  <si>
-    <t>10.10.10.10</t>
-  </si>
-  <si>
-    <t>TCP</t>
-  </si>
-  <si>
-    <t>UDP</t>
-  </si>
-  <si>
-    <t>*</t>
-  </si>
-  <si>
-    <t>CATCH_MISSED_TRAFFIC_TCP</t>
-  </si>
-  <si>
     <t>CATCH_MISSED_TRAFFIC_UDP</t>
   </si>
   <si>
-    <t>Permanent</t>
-  </si>
-  <si>
-    <t>Temporary Rule Duration (in Days)</t>
-  </si>
-  <si>
-    <t>Protection Rule</t>
-  </si>
-  <si>
-    <t>Default Rule to catch Missed Traffic TCP</t>
-  </si>
-  <si>
     <t>Default Rule to catch Missed Traffic UDP</t>
   </si>
   <si>
-    <t>CI20</t>
-  </si>
-  <si>
-    <t>CI40</t>
-  </si>
-  <si>
-    <t>CI50</t>
-  </si>
-  <si>
-    <t>hostname1.porche.com</t>
-  </si>
-  <si>
-    <t>hostname2.porche.com</t>
-  </si>
-  <si>
-    <t>hostname1.porche.com, hostname2.porche.com, hostname3.porche.com, hostname4.porche.com</t>
-  </si>
-  <si>
-    <t>10.10.10.10, 10.10.10.11, 10.10.10.12, 10.10.10.13, 10.10.10.14, 10.10.10.15</t>
-  </si>
-  <si>
-    <t>200.28.32.12,200.16.20.30,200.16.20.31, 200.16.20.32, 200.16.20.33, 200.16.20.34</t>
-  </si>
-  <si>
-    <t>1-65535;</t>
-  </si>
-  <si>
-    <t>10.200.0.0/16</t>
-  </si>
-  <si>
-    <t>60421; 1723; 33891; 25000; 49160; 8081; 12345; 53210; 4096; 650</t>
-  </si>
-  <si>
-    <t>32914;5872;44109;1023;65500;21345;38901;770-900;49152;12008</t>
-  </si>
-  <si>
-    <t>CI7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">hostname1.porche.com, </t>
-  </si>
-  <si>
-    <t>10.28.32.12,10.16.20.30,10.16.20.31, 10.16.20.32, 10.16.20.33,10.28.32.12, 10.16.20.34</t>
-  </si>
-  <si>
-    <t>Source IP address / Subnet / Range IP</t>
-  </si>
-  <si>
-    <t>Destination IP address / Subnet / Range IP</t>
-  </si>
-  <si>
-    <t>Hood_P_I_D</t>
-  </si>
-  <si>
-    <t>CI1 - Wheel_P</t>
-  </si>
-  <si>
-    <t>CI2 - Hood_P_I_D</t>
-  </si>
-  <si>
-    <t>CI4 - Wheel-New_1</t>
-  </si>
-  <si>
-    <t>CORE_Trunk_UDP</t>
-  </si>
-  <si>
-    <t>CORE_Fuel_UDP</t>
-  </si>
-  <si>
-    <t>CORE parts</t>
-  </si>
-  <si>
-    <t>Wheels_P</t>
-  </si>
-  <si>
-    <t>443,25;100;101</t>
-  </si>
-  <si>
-    <t>7878;8000</t>
-  </si>
-  <si>
-    <t>200.28.32.14,200.28.32.15</t>
-  </si>
-  <si>
-    <t>10.10.10.10, 10.10.10.11, 10.10.10.12</t>
-  </si>
-  <si>
-    <t>10.200.0.0/17</t>
-  </si>
-  <si>
-    <t>CORE_Speed_TCPPPPP</t>
-  </si>
-  <si>
-    <t>10.10.10.11</t>
-  </si>
-  <si>
-    <t>UPDATE</t>
-  </si>
-  <si>
-    <t>10.28.32.101</t>
-  </si>
-  <si>
-    <t>10.10.10.14</t>
-  </si>
-  <si>
-    <t>ANOTHER_NAME</t>
+    <r>
+      <t xml:space="preserve">10.10.10.10; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>28.32.15</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>200.28.32.12,200.16.20.30,200.16.20.31, 200.16.20.32, 200.16.20.33, 200.16.20.34</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -261,7 +375,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -271,6 +385,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -302,7 +422,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -313,7 +433,10 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -650,10 +773,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9AF1DFFD-6D3E-492F-B0C0-3C6733FA8AFB}">
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:O4"/>
   <sheetFormatPr defaultColWidth="21.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="6.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.77734375" customWidth="1"/>
     <col min="2" max="2" width="16.109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16.109375" customWidth="1"/>
     <col min="5" max="5" width="20" bestFit="1" customWidth="1"/>
@@ -666,159 +789,172 @@
     <col min="12" max="12" width="9.5546875" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="21.33203125" customWidth="1"/>
     <col min="14" max="14" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="18" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" s="1" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" s="1" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="3" t="s">
-        <v>44</v>
-      </c>
       <c r="D1" s="3" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>45</v>
+        <v>4</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="M1" s="3" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="N1" s="3" t="s">
-        <v>11</v>
+        <v>13</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="61.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:15" ht="61.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>36</v>
+        <v>17</v>
       </c>
       <c r="D2" s="2"/>
       <c r="E2" s="2" t="s">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="F2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G2" s="2" t="s">
         <v>20</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>40</v>
       </c>
       <c r="H2" s="2">
         <v>101</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="J2" s="2"/>
       <c r="K2" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="L2" s="2"/>
       <c r="M2" s="2" t="s">
-        <v>52</v>
+        <v>23</v>
       </c>
       <c r="N2" s="2"/>
+      <c r="O2" s="2"/>
     </row>
-    <row r="3" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B3" s="2" t="s">
+    <row r="3" spans="1:15" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D3" s="4"/>
+      <c r="E3" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G3" s="5">
+        <v>7878</v>
+      </c>
+      <c r="H3" s="4">
+        <v>103</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="J3" s="4"/>
+      <c r="K3" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="L3" s="4"/>
+      <c r="M3" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="N3" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="O3" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" ht="201.6" x14ac:dyDescent="0.3">
+      <c r="A4" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="F3" s="2" t="s">
+      <c r="C4" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="D4" s="4"/>
+      <c r="E4" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="G4" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="G3" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="H3" s="2">
-        <v>103</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="J3" s="2"/>
-      <c r="K3" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="L3" s="2"/>
-      <c r="M3" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="N3" s="2"/>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="H4" s="2">
+      <c r="H4" s="4">
         <v>104</v>
       </c>
-      <c r="I4" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="J4" s="2"/>
-      <c r="K4" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="L4" s="2"/>
-      <c r="M4" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="N4" s="2"/>
+      <c r="I4" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="J4" s="4"/>
+      <c r="K4" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="L4" s="4"/>
+      <c r="M4" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="N4" s="5"/>
+      <c r="O4" s="4" t="s">
+        <v>34</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
@@ -828,10 +964,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E6699DB-F1B6-43A3-AC90-D8377FCA7CDF}">
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:O7"/>
   <sheetFormatPr defaultColWidth="21.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="6.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="16.109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="28.5546875" customWidth="1"/>
     <col min="5" max="5" width="22.109375" customWidth="1"/>
@@ -843,255 +979,304 @@
     <col min="11" max="11" width="11.109375" customWidth="1"/>
     <col min="12" max="12" width="9.5546875" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="21.33203125" customWidth="1"/>
-    <col min="14" max="14" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="14" max="15" width="18.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" s="1" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" s="1" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="3" t="s">
-        <v>44</v>
-      </c>
       <c r="D1" s="3" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>45</v>
+        <v>4</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="M1" s="3" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="N1" s="3" t="s">
-        <v>11</v>
+        <v>13</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>13</v>
+        <v>35</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>17</v>
+        <v>36</v>
       </c>
       <c r="D2" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>19</v>
-      </c>
       <c r="G2" s="2" t="s">
-        <v>54</v>
+        <v>39</v>
       </c>
       <c r="H2" s="2">
         <v>1000</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>53</v>
+        <v>40</v>
       </c>
       <c r="J2" s="2"/>
       <c r="K2" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="L2" s="2"/>
       <c r="M2" s="2"/>
       <c r="N2" s="2" t="s">
-        <v>47</v>
-      </c>
+        <v>41</v>
+      </c>
+      <c r="O2" s="2"/>
     </row>
-    <row r="3" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:15" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>14</v>
+        <v>42</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>43</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="H3" s="2">
         <v>1001</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J3" s="2"/>
       <c r="K3" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="L3" s="2"/>
       <c r="M3" s="2"/>
       <c r="N3" s="2" t="s">
         <v>48</v>
       </c>
+      <c r="O3" s="2"/>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="G4" s="2">
-        <v>433</v>
+    <row r="4" spans="1:15" ht="244.8" x14ac:dyDescent="0.3">
+      <c r="A4" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>53</v>
       </c>
       <c r="H4" s="4">
         <v>1507</v>
       </c>
       <c r="I4" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="J4" s="4"/>
+      <c r="K4" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="L4" s="4"/>
+      <c r="M4" s="4"/>
+      <c r="N4" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="O4" s="4" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A5" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G5" s="4">
+        <v>433</v>
+      </c>
+      <c r="H5" s="4">
+        <v>1508</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="J5" s="4"/>
+      <c r="K5" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="L5" s="4"/>
+      <c r="M5" s="4"/>
+      <c r="N5" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="O5" s="4"/>
+    </row>
+    <row r="6" spans="1:15" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="E6" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="J4" s="2"/>
-      <c r="K4" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="L4" s="2"/>
-      <c r="M4" s="2"/>
-      <c r="N4" s="2" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H5" s="2">
+      <c r="F6" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="H6" s="2">
         <v>2001</v>
       </c>
-      <c r="I5" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="J5" s="2"/>
-      <c r="K5" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="L5" s="2">
-        <v>60</v>
-      </c>
-      <c r="M5" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="N5" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H6" s="2">
-        <v>2002</v>
-      </c>
       <c r="I6" s="2" t="s">
-        <v>23</v>
+        <v>65</v>
       </c>
       <c r="J6" s="2"/>
       <c r="K6" s="2" t="s">
-        <v>9</v>
+        <v>66</v>
       </c>
       <c r="L6" s="2">
         <v>60</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>28</v>
+        <v>67</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>26</v>
-      </c>
+        <v>68</v>
+      </c>
+      <c r="O6" s="2"/>
+    </row>
+    <row r="7" spans="1:15" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="H7" s="2">
+        <v>2002</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="J7" s="2"/>
+      <c r="K7" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="L7" s="2">
+        <v>60</v>
+      </c>
+      <c r="M7" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="N7" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="O7" s="2"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
 </file>
 
@@ -1105,6 +1290,14 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="28b9e305-6540-4a8f-adff-9abbf67a9457" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010015ACE1AB7268A5458AC0B83055E08635" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="e052996763366cd34d38aa15b997ceb6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="ca2eab16-4a02-4618-8f5f-796fd976fad0" xmlns:ns4="28b9e305-6540-4a8f-adff-9abbf67a9457" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9eb40f27300348baafeb0af7684f4cc8" ns3:_="" ns4:_="">
     <xsd:import namespace="ca2eab16-4a02-4618-8f5f-796fd976fad0"/>
@@ -1357,14 +1550,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="28b9e305-6540-4a8f-adff-9abbf67a9457" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D9D5B3E-6F96-42BC-A5EA-BACFD70EAC33}">
   <ds:schemaRefs>
@@ -1374,6 +1559,23 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{895FB154-B56A-495E-8783-E6DB4BCA3C3E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="ca2eab16-4a02-4618-8f5f-796fd976fad0"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="28b9e305-6540-4a8f-adff-9abbf67a9457"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4C515B5D-F162-4360-8913-11D1CBEB4EBF}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1392,23 +1594,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{895FB154-B56A-495E-8783-E6DB4BCA3C3E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="ca2eab16-4a02-4618-8f5f-796fd976fad0"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="28b9e305-6540-4a8f-adff-9abbf67a9457"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{94d26a2e-8b36-46ca-a6cf-bdb96546be89}" enabled="1" method="Privileged" siteId="{0b3fc178-b730-4e8b-9843-e81259237b77}" removed="0"/>

</xml_diff>